<commit_message>
Update dashboard styling and feed row rendering; stop tracking compiled Python cache
</commit_message>
<xml_diff>
--- a/risk_engine/config/fixed_mapping.xlsx
+++ b/risk_engine/config/fixed_mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/devjain/Downloads/erm2/risk_engine/config/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{E0B7DF54-CFD2-DF44-8689-5D3BEB1199BF}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2508299E-E6D6-BD45-A81E-D56C6475C3FA}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4440" yWindow="760" windowWidth="24960" windowHeight="17080" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1100" yWindow="760" windowWidth="24960" windowHeight="17080" activeTab="7" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Geopolitical_Mapping_v1" sheetId="1" r:id="rId1"/>
@@ -27,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="723" uniqueCount="209">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="687" uniqueCount="209">
   <si>
     <t>Structural Domain</t>
   </si>
@@ -1032,12 +1032,8 @@
       <c r="B1" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="C1" s="1" t="s">
-        <v>2</v>
-      </c>
-      <c r="D1" s="1" t="s">
-        <v>3</v>
-      </c>
+      <c r="C1" s="1"/>
+      <c r="D1" s="1"/>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
@@ -1046,12 +1042,6 @@
       <c r="B2" t="s">
         <v>5</v>
       </c>
-      <c r="C2" t="s">
-        <v>6</v>
-      </c>
-      <c r="D2" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
@@ -1060,12 +1050,6 @@
       <c r="B3" t="s">
         <v>6</v>
       </c>
-      <c r="C3" t="s">
-        <v>9</v>
-      </c>
-      <c r="D3" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
@@ -1074,12 +1058,6 @@
       <c r="B4" t="s">
         <v>5</v>
       </c>
-      <c r="C4" t="s">
-        <v>6</v>
-      </c>
-      <c r="D4" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A5" t="s">
@@ -1088,12 +1066,6 @@
       <c r="B5" t="s">
         <v>5</v>
       </c>
-      <c r="C5" t="s">
-        <v>6</v>
-      </c>
-      <c r="D5" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A6" t="s">
@@ -1102,12 +1074,6 @@
       <c r="B6" t="s">
         <v>5</v>
       </c>
-      <c r="C6" t="s">
-        <v>6</v>
-      </c>
-      <c r="D6" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A7" t="s">
@@ -1116,12 +1082,6 @@
       <c r="B7" t="s">
         <v>5</v>
       </c>
-      <c r="C7" t="s">
-        <v>6</v>
-      </c>
-      <c r="D7" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A8" t="s">
@@ -1130,12 +1090,6 @@
       <c r="B8" t="s">
         <v>5</v>
       </c>
-      <c r="C8" t="s">
-        <v>6</v>
-      </c>
-      <c r="D8" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A9" t="s">
@@ -1144,12 +1098,6 @@
       <c r="B9" t="s">
         <v>5</v>
       </c>
-      <c r="C9" t="s">
-        <v>6</v>
-      </c>
-      <c r="D9" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A10" t="s">
@@ -1158,12 +1106,6 @@
       <c r="B10" t="s">
         <v>5</v>
       </c>
-      <c r="C10" t="s">
-        <v>6</v>
-      </c>
-      <c r="D10" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A11" t="s">
@@ -1172,12 +1114,6 @@
       <c r="B11" t="s">
         <v>5</v>
       </c>
-      <c r="C11" t="s">
-        <v>6</v>
-      </c>
-      <c r="D11" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A12" t="s">
@@ -1186,12 +1122,6 @@
       <c r="B12" t="s">
         <v>5</v>
       </c>
-      <c r="C12" t="s">
-        <v>6</v>
-      </c>
-      <c r="D12" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A13" t="s">
@@ -1200,12 +1130,6 @@
       <c r="B13" t="s">
         <v>5</v>
       </c>
-      <c r="C13" t="s">
-        <v>6</v>
-      </c>
-      <c r="D13" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A14" t="s">
@@ -1214,12 +1138,6 @@
       <c r="B14" t="s">
         <v>7</v>
       </c>
-      <c r="C14" t="s">
-        <v>5</v>
-      </c>
-      <c r="D14" t="s">
-        <v>21</v>
-      </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A15" t="s">
@@ -1228,12 +1146,6 @@
       <c r="B15" t="s">
         <v>5</v>
       </c>
-      <c r="C15" t="s">
-        <v>6</v>
-      </c>
-      <c r="D15" t="s">
-        <v>7</v>
-      </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A16" t="s">
@@ -1242,42 +1154,24 @@
       <c r="B16" t="s">
         <v>5</v>
       </c>
-      <c r="C16" t="s">
-        <v>6</v>
-      </c>
-      <c r="D16" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="17" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="17" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A17" t="s">
         <v>24</v>
       </c>
       <c r="B17" t="s">
         <v>5</v>
       </c>
-      <c r="C17" t="s">
-        <v>6</v>
-      </c>
-      <c r="D17" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="18" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="18" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A18" t="s">
         <v>25</v>
       </c>
       <c r="B18" t="s">
         <v>5</v>
       </c>
-      <c r="C18" t="s">
-        <v>6</v>
-      </c>
-      <c r="D18" t="s">
-        <v>7</v>
-      </c>
-    </row>
-    <row r="19" spans="1:4" x14ac:dyDescent="0.2">
+    </row>
+    <row r="19" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A19" t="s">
         <v>27</v>
       </c>
@@ -1285,7 +1179,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="20" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="20" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A20" t="s">
         <v>29</v>
       </c>
@@ -1293,7 +1187,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="21" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="21" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A21" t="s">
         <v>31</v>
       </c>
@@ -1301,7 +1195,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="22" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="22" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A22" t="s">
         <v>33</v>
       </c>
@@ -1309,7 +1203,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="23" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="23" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A23" t="s">
         <v>35</v>
       </c>
@@ -1317,7 +1211,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="24" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="24" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A24" t="s">
         <v>37</v>
       </c>
@@ -1325,7 +1219,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="25" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="25" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A25" t="s">
         <v>39</v>
       </c>
@@ -1333,7 +1227,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="26" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A26" t="s">
         <v>41</v>
       </c>
@@ -1341,7 +1235,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="27" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="27" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A27" t="s">
         <v>43</v>
       </c>
@@ -1349,7 +1243,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="28" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="28" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A28" t="s">
         <v>45</v>
       </c>
@@ -1357,7 +1251,7 @@
         <v>5</v>
       </c>
     </row>
-    <row r="29" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="29" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A29" t="s">
         <v>47</v>
       </c>
@@ -1365,7 +1259,7 @@
         <v>7</v>
       </c>
     </row>
-    <row r="30" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="30" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A30" t="s">
         <v>49</v>
       </c>
@@ -1373,7 +1267,7 @@
         <v>6</v>
       </c>
     </row>
-    <row r="31" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="31" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A31" t="s">
         <v>53</v>
       </c>
@@ -1381,7 +1275,7 @@
         <v>21</v>
       </c>
     </row>
-    <row r="32" spans="1:4" x14ac:dyDescent="0.2">
+    <row r="32" spans="1:2" x14ac:dyDescent="0.2">
       <c r="A32" t="s">
         <v>56</v>
       </c>
@@ -1992,6 +1886,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="31" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="35" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
@@ -2515,7 +2410,9 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="45.5" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="103.83203125" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="28.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.2">
@@ -2818,6 +2715,7 @@
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="30.6640625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="106.6640625" bestFit="1" customWidth="1"/>
     <col min="3" max="3" width="21" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>

</xml_diff>